<commit_message>
Add admin announcements and pinning, Korean holiday classes, and configurable release time
</commit_message>
<xml_diff>
--- a/web/assets/onoff-workouts-example.xlsx
+++ b/web/assets/onoff-workouts-example.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="동작목록" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'수업등록'!$A$1:$H$1001</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'수업등록'!$A$1:$I$1001</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -447,6 +447,7 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -490,6 +491,11 @@
           <t>오늘 운동 설명 영상</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>수업 시간(공휴일)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -528,6 +534,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -568,6 +575,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="n"/>
     </row>
     <row r="4" ht="75" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -609,6 +617,7 @@
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="n"/>
     </row>
     <row r="5" ht="75" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -648,6 +657,7 @@
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="n"/>
     </row>
     <row r="6" ht="75" customHeight="1">
       <c r="A6" s="2" t="n"/>
@@ -658,6 +668,7 @@
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
     </row>
     <row r="7" ht="75" customHeight="1">
       <c r="A7" s="2" t="n"/>
@@ -668,6 +679,7 @@
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
     </row>
     <row r="8" ht="75" customHeight="1">
       <c r="A8" s="2" t="n"/>
@@ -678,6 +690,7 @@
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
     </row>
     <row r="9" ht="75" customHeight="1">
       <c r="A9" s="2" t="n"/>
@@ -688,6 +701,7 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
     </row>
     <row r="10" ht="75" customHeight="1">
       <c r="A10" s="2" t="n"/>
@@ -698,9 +712,10 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1001"/>
+  <autoFilter ref="A1:I1001"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="항목 확인" error="목록에서 선택해주세요." type="list">
       <formula1>"B/T,WOD"</formula1>
@@ -719,7 +734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -730,6 +745,7 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="75" customHeight="1">
@@ -773,6 +789,11 @@
           <t>오늘 운동 설명 영상</t>
         </is>
       </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>수업 시간(공휴일)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="75" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -811,6 +832,7 @@
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="n"/>
     </row>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -851,6 +873,7 @@
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="n"/>
     </row>
     <row r="4" ht="75" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -892,6 +915,7 @@
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="n"/>
     </row>
     <row r="5" ht="75" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -931,6 +955,7 @@
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -943,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -973,7 +998,7 @@
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>3. 수업: B/T 또는 WOD. 수요일은 WOD만, 토·일요일은 정규 수업을 등록하지 않습니다.</t>
+          <t>3. 수업: B/T 또는 WOD. 수요일은 WOD만, 토·일요일은 기본 휴강입니다. 공휴일 특별 수업은 수업 시간을 지정하세요.</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1047,7 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>10. 수업은 해당 날짜 전날 한국 시간 22:00에 자동 공개됩니다. 코치·운영자는 미리 볼 수 있습니다.</t>
+          <t>10. 수업은 해당 날짜 전날 운영자가 설정한 한국 시각에 자동 공개됩니다. 기본값은 22:00입니다. 코치·운영자는 미리 볼 수 있습니다.</t>
         </is>
       </c>
     </row>
@@ -1035,6 +1060,13 @@
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>공휴일 특별 수업: 수업 시간(공휴일) 열에 10:00, 11:00처럼 시작 시각을 입력합니다. 각 수업은 1시간입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>12. 예시파일은 기능 확인용입니다. 날짜와 내용을 실제 수업으로 바꾼 뒤 등록하세요.</t>
         </is>

</xml_diff>

<commit_message>
Streamline gym home, add personal 1RM catalogue and finalize login, identity and TV status
</commit_message>
<xml_diff>
--- a/web/assets/onoff-workouts-example.xlsx
+++ b/web/assets/onoff-workouts-example.xlsx
@@ -968,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1047,7 +1047,7 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>10. 수업은 해당 날짜 전날 운영자가 설정한 한국 시각에 자동 공개됩니다. 기본값은 22:00입니다. 코치·운영자는 미리 볼 수 있습니다.</t>
+          <t>10. 수업은 해당 날짜 전날 운영자가 설정한 한국 시각에 자동 공개됩니다. 기본값은 22:00입니다. 운영자는 미리 볼 수 있습니다.</t>
         </is>
       </c>
     </row>
@@ -1067,6 +1067,13 @@
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>추가 종목: 운영자가 앱에서 등록한 최신 종목 이름을 사용할 수 있습니다. 동작목록 시트는 기본 목록 참고용입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>12. 예시파일은 기능 확인용입니다. 날짜와 내용을 실제 수업으로 바꾼 뒤 등록하세요.</t>
         </is>
@@ -1083,7 +1090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1099,110 +1106,243 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Front Squat</t>
+          <t>Back Squat</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Back Squat</t>
+          <t>Front Squat</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Deadlift</t>
+          <t>Overhead Squat</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Clean</t>
+          <t>Shoulder Press</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Clean &amp; Jerk</t>
+          <t>Bench Press</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Snatch</t>
+          <t>Push Press</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Power Snatch</t>
+          <t>Push Jerk</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Squat Snatch</t>
+          <t>Split Jerk</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Strict Press</t>
+          <t>Deadlift</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Push Press</t>
+          <t>Sumo Deadlift</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Split Jerk</t>
+          <t>Power Clean</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Row</t>
+          <t>Squat Clean</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Box Step Over</t>
+          <t>Muscle Clean</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pull-up</t>
+          <t>Hang Power Clean</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ring Dip</t>
+          <t>Hang Squat Clean</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>Power Snatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Squat Snatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Muscle Snatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Hang Power Snatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Hang Squat Snatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Snatch Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Clean &amp; Jerk</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Clean &amp; Split Jerk</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Power Clean &amp; Jerk</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Power Clean &amp; Split Jerk</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Thruster</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Snatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Strict Press</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Box Step Over</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Pull-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Ring Dip</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Burpee</t>
         </is>

</xml_diff>